<commit_message>
Fix date issue in read_election_template function.
</commit_message>
<xml_diff>
--- a/tests/testthat/testdata/files_unparsed/election_templates/maj_template.xlsx
+++ b/tests/testthat/testdata/files_unparsed/election_templates/maj_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\STAT\01_Post\Graf\eCH-0157_testfiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\STAT\01_Post\Graf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2E78E8-7AAD-4FC8-A5A4-B552BF078419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B939E41-DDB9-44E2-BFFA-277F32FD5653}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="75" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="15" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="69">
   <si>
     <t>nachname</t>
   </si>
@@ -76,6 +76,33 @@
     <t>Marie</t>
   </si>
   <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>Kinderärztin, Praxisleiterin, Dr. med.</t>
+  </si>
+  <si>
+    <t>Hornbach</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Rheinau</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>ja</t>
+  </si>
+  <si>
+    <t>FDP</t>
+  </si>
+  <si>
+    <t>FDP.Die Liberalen</t>
+  </si>
+  <si>
     <t>Sägesser</t>
   </si>
   <si>
@@ -85,12 +112,48 @@
     <t>Ruedi</t>
   </si>
   <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>pensionierter Elektro-Ingenieur ETH, Jagdvorstand</t>
+  </si>
+  <si>
+    <t>Müllerstotz</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>GRÜNE</t>
+  </si>
+  <si>
     <t>Müller</t>
   </si>
   <si>
     <t>Fritz</t>
   </si>
   <si>
+    <t>Chauffeur</t>
+  </si>
+  <si>
+    <t>Dorfstrasse</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>EVP</t>
+  </si>
+  <si>
+    <t>Evangelische Volkspartei</t>
+  </si>
+  <si>
     <t>Opfiker</t>
   </si>
   <si>
@@ -100,151 +163,70 @@
     <t>Sandra</t>
   </si>
   <si>
+    <t>Käserin, EFZ</t>
+  </si>
+  <si>
+    <t>Seeblickstrasse</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>SVP</t>
+  </si>
+  <si>
+    <t>Schweizerische Volkspartei</t>
+  </si>
+  <si>
     <t>Pfister-Hauser</t>
   </si>
   <si>
     <t>Regula</t>
   </si>
   <si>
+    <t>Primarlehrerin, Heilpädagogin, Pilzexpertin</t>
+  </si>
+  <si>
+    <t>Dr.</t>
+  </si>
+  <si>
+    <t>Hermanngasse</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>Sozialdemokratische Partei</t>
+  </si>
+  <si>
     <t>Trub</t>
   </si>
   <si>
     <t>Samuel</t>
   </si>
   <si>
-    <t>1996-05-11</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>Kinderärztin, Praxisleiterin, Dr. med.</t>
-  </si>
-  <si>
-    <t>1956-10-21</t>
-  </si>
-  <si>
-    <t>pensionierter Elektro-Ingenieur ETH, Jagdvorstand</t>
-  </si>
-  <si>
-    <t>2000-03-02</t>
-  </si>
-  <si>
-    <t>Chauffeur</t>
-  </si>
-  <si>
-    <t>1978-12-06</t>
-  </si>
-  <si>
-    <t>Käserin, EFZ</t>
-  </si>
-  <si>
-    <t>1981-09-06</t>
-  </si>
-  <si>
-    <t>Primarlehrerin, Heilpädagogin, Pilzexpertin</t>
-  </si>
-  <si>
-    <t>1990-11-19</t>
-  </si>
-  <si>
     <t>Chemielaborant</t>
   </si>
   <si>
-    <t>Hornbach</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>Müllerstotz</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>Dorfstrasse</t>
-  </si>
-  <si>
-    <t>120</t>
-  </si>
-  <si>
-    <t>Seeblickstrasse</t>
-  </si>
-  <si>
-    <t>Hermanngasse</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
     <t>Pfingstweid</t>
   </si>
   <si>
     <t>6</t>
   </si>
   <si>
-    <t>Rheinau</t>
-  </si>
-  <si>
-    <t>FDP</t>
-  </si>
-  <si>
-    <t>FDP.Die Liberalen</t>
-  </si>
-  <si>
-    <t>GRÜNE</t>
-  </si>
-  <si>
-    <t>EVP</t>
-  </si>
-  <si>
-    <t>Evangelische Volkspartei</t>
-  </si>
-  <si>
-    <t>SVP</t>
-  </si>
-  <si>
-    <t>Schweizerische Volkspartei</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>Sozialdemokratische Partei</t>
+    <t>06</t>
   </si>
   <si>
     <t>parteilos</t>
-  </si>
-  <si>
-    <t>Dr.</t>
-  </si>
-  <si>
-    <t>ja</t>
-  </si>
-  <si>
-    <t>w</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>05</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>06</t>
   </si>
 </sst>
 </file>
@@ -288,11 +270,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -610,7 +594,7 @@
     <col min="8" max="8" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -674,79 +658,79 @@
       <c r="C2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" t="s">
-        <v>30</v>
+      <c r="D2" s="2">
+        <v>35196</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="I2" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="J2">
         <v>8464</v>
       </c>
       <c r="K2" t="s">
-        <v>54</v>
-      </c>
-      <c r="L2" t="s">
-        <v>69</v>
+        <v>22</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="M2" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="N2" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="O2" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="2">
+        <v>20749</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
         <v>33</v>
-      </c>
-      <c r="E3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H3" t="s">
-        <v>45</v>
-      </c>
-      <c r="I3" t="s">
-        <v>46</v>
       </c>
       <c r="J3">
         <v>8464</v>
       </c>
       <c r="K3" t="s">
-        <v>54</v>
-      </c>
-      <c r="L3" t="s">
-        <v>70</v>
+        <v>22</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="N3" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="O3" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -759,255 +743,255 @@
       <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" t="s">
-        <v>30</v>
+      <c r="D4" s="2">
+        <v>35196</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="H4" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="I4" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="J4">
         <v>8464</v>
       </c>
       <c r="K4" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="L4" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="M4" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="N4" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="O4" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="D5" s="2">
+        <v>36587</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H5" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="I5" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="J5">
         <v>8464</v>
       </c>
       <c r="K5" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="L5" t="s">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="M5" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="N5" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="O5" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" t="s">
-        <v>37</v>
+        <v>46</v>
+      </c>
+      <c r="D6" s="2">
+        <v>28830</v>
       </c>
       <c r="E6" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="H6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" t="s">
         <v>49</v>
-      </c>
-      <c r="I6" t="s">
-        <v>31</v>
       </c>
       <c r="J6">
         <v>8464</v>
       </c>
       <c r="K6" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="L6" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="M6" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="N6" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="O6" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>39</v>
+        <v>54</v>
+      </c>
+      <c r="D7" s="2">
+        <v>29835</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="G7" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="H7" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="I7" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="J7">
         <v>8464</v>
       </c>
       <c r="K7" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="L7" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="N7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="2">
+        <v>20749</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
         <v>33</v>
-      </c>
-      <c r="E8" t="s">
-        <v>68</v>
-      </c>
-      <c r="F8" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" t="s">
-        <v>45</v>
-      </c>
-      <c r="I8" t="s">
-        <v>46</v>
       </c>
       <c r="J8">
         <v>8464</v>
       </c>
       <c r="K8" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="L8" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="M8" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="N8" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="O8" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" t="s">
-        <v>41</v>
+        <v>63</v>
+      </c>
+      <c r="D9" s="2">
+        <v>33196</v>
       </c>
       <c r="E9" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="I9" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="J9">
         <v>8464</v>
       </c>
       <c r="K9" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="L9" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="N9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="O9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>